<commit_message>
updated cal sheet with data from CultureCronulla experiment
</commit_message>
<xml_diff>
--- a/calibration/calibration_sheet.xlsx
+++ b/calibration/calibration_sheet.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngdan\Documents\WhaleX\AquaPi\aqua-pi-live\aqua-pi\calibration\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ngdan\Documents\aquapi-live\aquapi\calibration\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BB814FBE-20B1-48BB-B1B3-F7FE96C3F1F4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA5D4E0-C88B-47D1-90EA-0680F7D25A29}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" firstSheet="1" activeTab="10" xr2:uid="{F5773221-019F-4E21-9389-E209F6CA127D}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" firstSheet="6" activeTab="10" xr2:uid="{F5773221-019F-4E21-9389-E209F6CA127D}"/>
   </bookViews>
   <sheets>
     <sheet name="calibrations oct-2024" sheetId="1" r:id="rId1"/>
@@ -29,6 +29,7 @@
     <externalReference r:id="rId12"/>
   </externalReferences>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -49,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="672" uniqueCount="127">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="673" uniqueCount="128">
   <si>
     <t xml:space="preserve">Blank </t>
   </si>
@@ -432,6 +433,9 @@
   <si>
     <t>AP01GAIN</t>
   </si>
+  <si>
+    <t>u</t>
+  </si>
 </sst>
 </file>
 
@@ -454,18 +458,12 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFFF00"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="1">
@@ -480,7 +478,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="22" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
@@ -490,7 +488,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1424,7 +1421,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -1870,7 +1867,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -1993,7 +1990,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2160,7 +2157,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -2486,7 +2483,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2609,7 +2606,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -2784,7 +2781,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -3350,7 +3347,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -3473,7 +3470,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -4174,7 +4171,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -4640,7 +4637,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -4763,7 +4760,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -4946,7 +4943,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -5260,7 +5257,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -5383,7 +5380,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -5566,7 +5563,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -6150,7 +6147,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -6273,7 +6270,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -6974,7 +6971,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -7300,7 +7297,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -7423,7 +7420,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -7912,7 +7909,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -8352,7 +8349,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -8475,7 +8472,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -8658,7 +8655,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -9218,7 +9215,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -9341,7 +9338,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -9542,13 +9539,13 @@
                   <c:v>236.37455830388598</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>99.80753920134768</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>99.80753920134768</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>99.80753920134768</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -9912,13 +9909,13 @@
                   <c:v>272.45999999999998</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>144.55148816659079</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>144.55148816659079</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>144.55148816659079</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10304,13 +10301,13 @@
                   <c:v>228.36276595744599</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>140.13157145734613</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>140.13157145734613</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>20</c:v>
+                  <c:v>140.13157145734613</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -10696,13 +10693,13 @@
                   <c:v>822.87588652482202</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>99.80753920134768</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>99.80753920134768</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>99.80753920134768</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11092,13 +11089,13 @@
                   <c:v>1010.11851851851</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0</c:v>
+                  <c:v>144.55148816659079</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0</c:v>
+                  <c:v>144.55148816659079</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0</c:v>
+                  <c:v>144.55148816659079</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -11484,13 +11481,13 @@
                   <c:v>830.899224806201</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>20</c:v>
+                  <c:v>140.13157145734613</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>20</c:v>
+                  <c:v>140.13157145734613</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>20</c:v>
+                  <c:v>140.13157145734613</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -12081,7 +12078,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -12407,7 +12404,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -12530,7 +12527,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -12713,7 +12710,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -13159,7 +13156,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13282,7 +13279,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -13465,7 +13462,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -13931,7 +13928,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -14054,7 +14051,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -14237,7 +14234,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -14551,7 +14548,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -14674,7 +14671,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -14857,7 +14854,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -15183,7 +15180,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -15306,7 +15303,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -15489,7 +15486,7 @@
               <a:cs typeface="+mn-cs"/>
             </a:defRPr>
           </a:pPr>
-          <a:endParaRPr lang="en-AU"/>
+          <a:endParaRPr lang="en-US"/>
         </a:p>
       </c:txPr>
     </c:title>
@@ -15929,7 +15926,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -16052,7 +16049,7 @@
                   <a:cs typeface="+mn-cs"/>
                 </a:defRPr>
               </a:pPr>
-              <a:endParaRPr lang="en-AU"/>
+              <a:endParaRPr lang="en-US"/>
             </a:p>
           </c:txPr>
         </c:title>
@@ -30320,16 +30317,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6B211761-E504-431E-93E2-CFA7BCB34520}">
   <dimension ref="A1:H4"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="24.140625" customWidth="1"/>
-    <col min="2" max="2" width="38.140625" customWidth="1"/>
-    <col min="3" max="3" width="18.28515625" customWidth="1"/>
+    <col min="1" max="1" width="24.1796875" customWidth="1"/>
+    <col min="2" max="2" width="38.1796875" customWidth="1"/>
+    <col min="3" max="3" width="18.26953125" customWidth="1"/>
     <col min="4" max="4" width="15" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.54296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>1</v>
       </c>
@@ -30352,7 +30349,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>2</v>
       </c>
@@ -30377,7 +30374,7 @@
         <v>45566</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>59</v>
       </c>
@@ -30389,7 +30386,7 @@
         <v>2020.8</v>
       </c>
       <c r="D3">
-        <f t="shared" ref="D3:D4" si="0">40/C3</f>
+        <f>40/C3</f>
         <v>1.9794140934283451E-2</v>
       </c>
       <c r="E3" t="s">
@@ -30402,7 +30399,7 @@
         <v>45566</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>60</v>
       </c>
@@ -30414,7 +30411,7 @@
         <v>2662.5</v>
       </c>
       <c r="D4">
-        <f t="shared" si="0"/>
+        <f>40/C4</f>
         <v>1.5023474178403756E-2</v>
       </c>
       <c r="E4" t="s">
@@ -30435,7 +30432,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C54D3315-7263-483B-AAE2-A8D960C073F8}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -30443,14 +30440,14 @@
 
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48340B77-1A63-44BB-9167-6E7FB155313D}">
-  <dimension ref="A1:Z10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <dimension ref="A1:Z12"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="2" width="19.140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="11" width="22.42578125" customWidth="1"/>
+    <col min="1" max="2" width="19.1796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="11" width="22.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>107</v>
       </c>
@@ -30485,7 +30482,7 @@
         <v>125</v>
       </c>
     </row>
-    <row r="2" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A2" t="s">
         <v>114</v>
       </c>
@@ -30527,7 +30524,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="3" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A3" t="s">
         <v>116</v>
       </c>
@@ -30569,7 +30566,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="4" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A4" t="s">
         <v>117</v>
       </c>
@@ -30611,7 +30608,7 @@
         <v>200</v>
       </c>
     </row>
-    <row r="5" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A5" t="s">
         <v>118</v>
       </c>
@@ -30622,7 +30619,7 @@
         <v>2286.0992907801401</v>
       </c>
       <c r="D5">
-        <f>C5/10</f>
+        <f t="shared" ref="D5:D10" si="1">C5/10</f>
         <v>228.60992907801401</v>
       </c>
       <c r="E5" t="s">
@@ -30632,7 +30629,7 @@
         <v>2731.93307086614</v>
       </c>
       <c r="G5">
-        <f>F5/10</f>
+        <f t="shared" ref="G5:G10" si="2">F5/10</f>
         <v>273.19330708661403</v>
       </c>
       <c r="H5" t="s">
@@ -30642,7 +30639,7 @@
         <v>2359.6868327402099</v>
       </c>
       <c r="J5">
-        <f>I5/10</f>
+        <f t="shared" ref="J5:J10" si="3">I5/10</f>
         <v>235.96868327402098</v>
       </c>
       <c r="K5" t="s">
@@ -30656,7 +30653,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="6" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A6" t="s">
         <v>119</v>
       </c>
@@ -30667,7 +30664,7 @@
         <v>2287.8915662650502</v>
       </c>
       <c r="D6">
-        <f>C6/10</f>
+        <f t="shared" si="1"/>
         <v>228.78915662650502</v>
       </c>
       <c r="E6" t="s">
@@ -30677,7 +30674,7 @@
         <v>2726.2401433691698</v>
       </c>
       <c r="G6">
-        <f t="shared" ref="G6:G10" si="1">F6/10</f>
+        <f t="shared" si="2"/>
         <v>272.62401433691696</v>
       </c>
       <c r="H6" t="s">
@@ -30687,7 +30684,7 @@
         <v>2364.3688524590102</v>
       </c>
       <c r="J6">
-        <f t="shared" ref="J6:J10" si="2">I6/10</f>
+        <f t="shared" si="3"/>
         <v>236.43688524590101</v>
       </c>
       <c r="K6" t="s">
@@ -30716,7 +30713,7 @@
         <v>106</v>
       </c>
     </row>
-    <row r="7" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A7" t="s">
         <v>120</v>
       </c>
@@ -30727,7 +30724,7 @@
         <v>2283.6276595744598</v>
       </c>
       <c r="D7">
-        <f>C7/10</f>
+        <f t="shared" si="1"/>
         <v>228.36276595744599</v>
       </c>
       <c r="E7" t="s">
@@ -30737,7 +30734,7 @@
         <v>2724.6</v>
       </c>
       <c r="G7">
-        <f t="shared" si="1"/>
+        <f t="shared" si="2"/>
         <v>272.45999999999998</v>
       </c>
       <c r="H7" t="s">
@@ -30747,7 +30744,7 @@
         <v>2363.7455830388599</v>
       </c>
       <c r="J7">
-        <f t="shared" si="2"/>
+        <f t="shared" si="3"/>
         <v>236.37455830388598</v>
       </c>
       <c r="K7" t="s">
@@ -30778,32 +30775,36 @@
         <v>187.5</v>
       </c>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>124</v>
       </c>
-      <c r="C8" s="7">
-        <v>200</v>
+      <c r="C8">
+        <v>1401.3157145734613</v>
       </c>
       <c r="D8">
-        <f>C8/10</f>
-        <v>20</v>
+        <f t="shared" si="1"/>
+        <v>140.13157145734613</v>
       </c>
       <c r="E8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F8" s="7"/>
+      <c r="F8">
+        <v>1445.514881665908</v>
+      </c>
       <c r="G8">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>144.55148816659079</v>
       </c>
       <c r="H8" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I8" s="7"/>
+      <c r="I8">
+        <v>998.07539201347674</v>
+      </c>
       <c r="J8">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>99.80753920134768</v>
       </c>
       <c r="K8" s="3" t="s">
         <v>72</v>
@@ -30832,32 +30833,36 @@
         <v>187.5</v>
       </c>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A9" t="s">
         <v>124</v>
       </c>
-      <c r="C9" s="7">
-        <v>200</v>
+      <c r="C9">
+        <v>1401.3157145734613</v>
       </c>
       <c r="D9">
-        <f>C9/10</f>
-        <v>20</v>
+        <f t="shared" si="1"/>
+        <v>140.13157145734613</v>
       </c>
       <c r="E9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F9" s="7"/>
+      <c r="F9">
+        <v>1445.514881665908</v>
+      </c>
       <c r="G9">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>144.55148816659079</v>
       </c>
       <c r="H9" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I9" s="7"/>
+      <c r="I9">
+        <v>998.07539201347674</v>
+      </c>
       <c r="J9">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>99.80753920134768</v>
       </c>
       <c r="K9" s="3" t="s">
         <v>72</v>
@@ -30870,32 +30875,36 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>124</v>
       </c>
-      <c r="C10" s="7">
-        <v>200</v>
+      <c r="C10">
+        <v>1401.3157145734613</v>
       </c>
       <c r="D10">
-        <f>C10/10</f>
-        <v>20</v>
+        <f t="shared" si="1"/>
+        <v>140.13157145734613</v>
       </c>
       <c r="E10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="F10" s="7"/>
+      <c r="F10">
+        <v>1445.514881665908</v>
+      </c>
       <c r="G10">
-        <f t="shared" si="1"/>
-        <v>0</v>
+        <f t="shared" si="2"/>
+        <v>144.55148816659079</v>
       </c>
       <c r="H10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="I10" s="7"/>
+      <c r="I10">
+        <v>998.07539201347674</v>
+      </c>
       <c r="J10">
-        <f t="shared" si="2"/>
-        <v>0</v>
+        <f t="shared" si="3"/>
+        <v>99.80753920134768</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>72</v>
@@ -30906,6 +30915,11 @@
       </c>
       <c r="M10">
         <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:26" x14ac:dyDescent="0.35">
+      <c r="R12" t="s">
+        <v>127</v>
       </c>
     </row>
   </sheetData>
@@ -30917,14 +30931,14 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{89BF18F8-9EF1-41BD-9E4E-C22057B73A82}">
   <dimension ref="A1:T46"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="12.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.28515625" customWidth="1"/>
-    <col min="7" max="7" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.26953125" customWidth="1"/>
+    <col min="7" max="7" width="11.7265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>93</v>
       </c>
@@ -30953,7 +30967,7 @@
         <v>93</v>
       </c>
     </row>
-    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>30</v>
       </c>
@@ -30982,7 +30996,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B3">
         <v>1</v>
       </c>
@@ -31008,7 +31022,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B4">
         <v>1</v>
       </c>
@@ -31034,7 +31048,7 @@
         <v>19.25</v>
       </c>
     </row>
-    <row r="5" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B5">
         <v>2</v>
       </c>
@@ -31063,7 +31077,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B6">
         <v>2</v>
       </c>
@@ -31077,7 +31091,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="7" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B7">
         <v>2</v>
       </c>
@@ -31091,7 +31105,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="8" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B8">
         <v>3</v>
       </c>
@@ -31102,7 +31116,7 @@
         <v>2063.3000000000002</v>
       </c>
     </row>
-    <row r="9" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B9">
         <v>3</v>
       </c>
@@ -31113,7 +31127,7 @@
         <v>2062.8000000000002</v>
       </c>
     </row>
-    <row r="10" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:11" x14ac:dyDescent="0.35">
       <c r="B10">
         <v>3</v>
       </c>
@@ -31124,7 +31138,7 @@
         <v>2062.5</v>
       </c>
     </row>
-    <row r="11" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>41.024999999999999</v>
       </c>
@@ -31138,7 +31152,7 @@
         <v>2300.1999999999998</v>
       </c>
     </row>
-    <row r="12" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A12">
         <v>41.024999999999999</v>
       </c>
@@ -31152,7 +31166,7 @@
         <v>2298.6999999999998</v>
       </c>
     </row>
-    <row r="13" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>41.024999999999999</v>
       </c>
@@ -31166,7 +31180,7 @@
         <v>2299.6</v>
       </c>
     </row>
-    <row r="14" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>41.024999999999999</v>
       </c>
@@ -31180,7 +31194,7 @@
         <v>2334.6</v>
       </c>
     </row>
-    <row r="15" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>41.024999999999999</v>
       </c>
@@ -31194,7 +31208,7 @@
         <v>2336.5</v>
       </c>
     </row>
-    <row r="16" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:11" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>41.024999999999999</v>
       </c>
@@ -31208,7 +31222,7 @@
         <v>2337.1999999999998</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>41.024999999999999</v>
       </c>
@@ -31222,7 +31236,7 @@
         <v>2280.6999999999998</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>41.024999999999999</v>
       </c>
@@ -31236,7 +31250,7 @@
         <v>2278.8000000000002</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>41.024999999999999</v>
       </c>
@@ -31250,7 +31264,7 @@
         <v>2279.1</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>26</v>
       </c>
@@ -31264,7 +31278,7 @@
         <v>1989.1</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>26</v>
       </c>
@@ -31278,7 +31292,7 @@
         <v>1989.4</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>26</v>
       </c>
@@ -31292,7 +31306,7 @@
         <v>1989.5</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>26</v>
       </c>
@@ -31306,7 +31320,7 @@
         <v>2015</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>26</v>
       </c>
@@ -31320,7 +31334,7 @@
         <v>2014.2</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>26</v>
       </c>
@@ -31334,7 +31348,7 @@
         <v>2015.8</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>26</v>
       </c>
@@ -31348,7 +31362,7 @@
         <v>1966.4</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>26</v>
       </c>
@@ -31362,7 +31376,7 @@
         <v>1966.4</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>26</v>
       </c>
@@ -31376,7 +31390,7 @@
         <v>1966.4</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>19.25</v>
       </c>
@@ -31390,7 +31404,7 @@
         <v>1806.7</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B30">
         <v>1</v>
       </c>
@@ -31401,7 +31415,7 @@
         <v>1808.2</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.35">
       <c r="B31">
         <v>1</v>
       </c>
@@ -31412,7 +31426,7 @@
         <v>1807.4</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>19.25</v>
       </c>
@@ -31426,7 +31440,7 @@
         <v>1825</v>
       </c>
     </row>
-    <row r="33" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B33">
         <v>2</v>
       </c>
@@ -31437,7 +31451,7 @@
         <v>1824.7</v>
       </c>
     </row>
-    <row r="34" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B34">
         <v>2</v>
       </c>
@@ -31448,7 +31462,7 @@
         <v>1824.6</v>
       </c>
     </row>
-    <row r="35" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>19.25</v>
       </c>
@@ -31462,7 +31476,7 @@
         <v>1784.7</v>
       </c>
     </row>
-    <row r="36" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B36">
         <v>3</v>
       </c>
@@ -31473,7 +31487,7 @@
         <v>1783.5</v>
       </c>
     </row>
-    <row r="37" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B37">
         <v>3</v>
       </c>
@@ -31487,7 +31501,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="38" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>15</v>
       </c>
@@ -31501,7 +31515,7 @@
         <v>1677.8</v>
       </c>
     </row>
-    <row r="39" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B39">
         <v>1</v>
       </c>
@@ -31512,7 +31526,7 @@
         <v>1678.6</v>
       </c>
     </row>
-    <row r="40" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B40">
         <v>1</v>
       </c>
@@ -31523,7 +31537,7 @@
         <v>1679.1</v>
       </c>
     </row>
-    <row r="41" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>15</v>
       </c>
@@ -31537,7 +31551,7 @@
         <v>1689.2</v>
       </c>
     </row>
-    <row r="42" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B42">
         <v>2</v>
       </c>
@@ -31548,7 +31562,7 @@
         <v>1690.2</v>
       </c>
     </row>
-    <row r="43" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B43">
         <v>2</v>
       </c>
@@ -31562,7 +31576,7 @@
         <v>101</v>
       </c>
     </row>
-    <row r="44" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>15</v>
       </c>
@@ -31576,7 +31590,7 @@
         <v>1653.4</v>
       </c>
     </row>
-    <row r="45" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B45">
         <v>3</v>
       </c>
@@ -31587,7 +31601,7 @@
         <v>1652.9</v>
       </c>
     </row>
-    <row r="46" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" x14ac:dyDescent="0.35">
       <c r="B46">
         <v>3</v>
       </c>
@@ -31607,12 +31621,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{713D51AC-D38B-4CEF-B4B9-2FA14F90FF6C}">
   <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="27.7109375" customWidth="1"/>
+    <col min="1" max="1" width="27.7265625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -31674,7 +31688,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45582.733738425923</v>
       </c>
@@ -31736,7 +31750,7 @@
         <v>6.86</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45582.7341087963</v>
       </c>
@@ -31798,7 +31812,7 @@
         <v>6.7751999999999999</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45582.734467592592</v>
       </c>
@@ -31860,7 +31874,7 @@
         <v>6.7857999999999903</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45582.734826388885</v>
       </c>
@@ -31922,7 +31936,7 @@
         <v>6.6585999999999999</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45582.735196759262</v>
       </c>
@@ -31984,7 +31998,7 @@
         <v>6.7539999999999996</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45582.735567129632</v>
       </c>
@@ -32046,7 +32060,7 @@
         <v>6.8281999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>45582.735925925925</v>
       </c>
@@ -32108,7 +32122,7 @@
         <v>6.7645999999999997</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>45582.736273148148</v>
       </c>
@@ -32170,7 +32184,7 @@
         <v>6.6797999999999904</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>45582.736643518518</v>
       </c>
@@ -32232,7 +32246,7 @@
         <v>6.9554</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>45582.737002314818</v>
       </c>
@@ -32302,12 +32316,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F68836B1-1488-4876-9A64-AECEECB061CE}">
   <dimension ref="A1:T11"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="29.28515625" customWidth="1"/>
+    <col min="1" max="1" width="29.26953125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -32369,7 +32383,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45582.748414351852</v>
       </c>
@@ -32431,7 +32445,7 @@
         <v>7.1143999999999998</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45582.748773148145</v>
       </c>
@@ -32493,7 +32507,7 @@
         <v>7.0720000000000001</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45582.749178240738</v>
       </c>
@@ -32555,7 +32569,7 @@
         <v>7.0613999999999999</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45582.749606481484</v>
       </c>
@@ -32617,7 +32631,7 @@
         <v>7.0295999999999896</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45582.750300925924</v>
       </c>
@@ -32679,7 +32693,7 @@
         <v>7.1249999999999902</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45582.751354166663</v>
       </c>
@@ -32741,7 +32755,7 @@
         <v>6.8811999999999998</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>45582.752256944441</v>
       </c>
@@ -32803,7 +32817,7 @@
         <v>6.8705999999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>45582.752962962964</v>
       </c>
@@ -32865,7 +32879,7 @@
         <v>6.8281999999999998</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>45582.753668981481</v>
       </c>
@@ -32927,7 +32941,7 @@
         <v>6.7434000000000003</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>45582.754374999997</v>
       </c>
@@ -32997,12 +33011,12 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A49D5A92-C4FB-4266-AFA3-C6B72E7BF3DD}">
   <dimension ref="A1:T16"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="35.85546875" customWidth="1"/>
+    <col min="1" max="1" width="35.81640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>37</v>
       </c>
@@ -33064,7 +33078,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="2" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>45582.804270833331</v>
       </c>
@@ -33117,7 +33131,7 @@
         <v>13.3154</v>
       </c>
     </row>
-    <row r="3" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>45582.804618055554</v>
       </c>
@@ -33170,7 +33184,7 @@
         <v>7.0507999999999997</v>
       </c>
     </row>
-    <row r="4" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>45582.805335648147</v>
       </c>
@@ -33223,7 +33237,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>45582.805590277778</v>
       </c>
@@ -33276,7 +33290,7 @@
         <v>7.0932000000000004</v>
       </c>
     </row>
-    <row r="6" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>45582.805856481478</v>
       </c>
@@ -33329,7 +33343,7 @@
         <v>13.962</v>
       </c>
     </row>
-    <row r="7" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>45582.806388888886</v>
       </c>
@@ -33382,7 +33396,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="8" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A8" s="1">
         <v>45582.80672453704</v>
       </c>
@@ -33435,7 +33449,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="9" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A9" s="1">
         <v>45582.808541666665</v>
       </c>
@@ -33488,7 +33502,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="10" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A10" s="1">
         <v>45582.809305555558</v>
       </c>
@@ -33541,7 +33555,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="11" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A11" s="1">
         <v>45582.815324074072</v>
       </c>
@@ -33594,7 +33608,7 @@
         <v>12.1812</v>
       </c>
     </row>
-    <row r="12" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>45582.815844907411</v>
       </c>
@@ -33647,7 +33661,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="13" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A13" s="1">
         <v>45582.816608796296</v>
       </c>
@@ -33700,7 +33714,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="14" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A14" s="1">
         <v>45582.81695601852</v>
       </c>
@@ -33753,7 +33767,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="16" spans="1:20" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" x14ac:dyDescent="0.35">
       <c r="K16">
         <f>AVERAGE(K2:K12)</f>
         <v>838.90909090909088</v>
@@ -33768,16 +33782,16 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DA1BF182-5206-4256-9322-E65B830D2C68}">
   <dimension ref="A1:H10"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="20.140625" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="20.1796875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="12.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="46.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="37.140625" customWidth="1"/>
+    <col min="4" max="4" width="12.7265625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="46.7265625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="37.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>92</v>
       </c>
@@ -33800,7 +33814,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B2" t="s">
         <v>80</v>
       </c>
@@ -33821,7 +33835,7 @@
         <v>38.0005427838</v>
       </c>
     </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C3">
         <v>2.6735410500000001E-2</v>
       </c>
@@ -33842,7 +33856,7 @@
         <v>38.0005427838</v>
       </c>
     </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C4">
         <v>2.3069651900000002E-2</v>
       </c>
@@ -33863,7 +33877,7 @@
         <v>34.323967228400001</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B5" t="s">
         <v>81</v>
       </c>
@@ -33887,7 +33901,7 @@
         <v>30.283843940300002</v>
       </c>
     </row>
-    <row r="6" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="C6">
         <v>2.0155495700000001E-2</v>
       </c>
@@ -33908,7 +33922,7 @@
         <v>30.283843940300002</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="30" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="29" x14ac:dyDescent="0.35">
       <c r="C7">
         <v>1.8836572199999999E-2</v>
       </c>
@@ -33929,7 +33943,7 @@
         <v>28.153738842599999</v>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" x14ac:dyDescent="0.35">
       <c r="B8" t="s">
         <v>78</v>
       </c>
@@ -33953,7 +33967,7 @@
         <v>40.744719201099997</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C9">
         <v>3.2164137199999998E-2</v>
       </c>
@@ -33974,7 +33988,7 @@
         <v>40.744719201099997</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="C10">
         <v>2.9297702700000001E-2</v>
       </c>
@@ -34004,18 +34018,18 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9C595185-4E42-455E-BD84-87D52B1BBF0F}">
   <dimension ref="A1:J61"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>66</v>
       </c>
@@ -34047,7 +34061,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>800</v>
       </c>
@@ -34081,7 +34095,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>800</v>
       </c>
@@ -34115,7 +34129,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>800</v>
       </c>
@@ -34149,7 +34163,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>800</v>
       </c>
@@ -34183,7 +34197,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>800</v>
       </c>
@@ -34217,7 +34231,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
         <f>A2/2</f>
         <v>400</v>
@@ -34252,7 +34266,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
         <f t="shared" ref="A8:A35" si="2">A3/2</f>
         <v>400</v>
@@ -34287,7 +34301,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
         <f t="shared" si="2"/>
         <v>400</v>
@@ -34322,7 +34336,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
         <f t="shared" si="2"/>
         <v>400</v>
@@ -34357,7 +34371,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
         <f t="shared" si="2"/>
         <v>400</v>
@@ -34392,7 +34406,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -34427,7 +34441,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -34462,7 +34476,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -34497,7 +34511,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -34532,7 +34546,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <f t="shared" si="2"/>
         <v>200</v>
@@ -34567,7 +34581,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <f t="shared" si="2"/>
         <v>100</v>
@@ -34602,7 +34616,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <f t="shared" si="2"/>
         <v>100</v>
@@ -34637,7 +34651,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <f t="shared" si="2"/>
         <v>100</v>
@@ -34672,7 +34686,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <f t="shared" si="2"/>
         <v>100</v>
@@ -34707,7 +34721,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <f t="shared" si="2"/>
         <v>100</v>
@@ -34742,7 +34756,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <f t="shared" si="2"/>
         <v>50</v>
@@ -34777,7 +34791,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <f t="shared" si="2"/>
         <v>50</v>
@@ -34812,7 +34826,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <f t="shared" si="2"/>
         <v>50</v>
@@ -34847,7 +34861,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <f t="shared" si="2"/>
         <v>50</v>
@@ -34882,7 +34896,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <f t="shared" si="2"/>
         <v>50</v>
@@ -34917,7 +34931,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -34952,7 +34966,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -34987,7 +35001,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -35022,7 +35036,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -35057,7 +35071,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <f t="shared" si="2"/>
         <v>25</v>
@@ -35092,7 +35106,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <f t="shared" si="2"/>
         <v>12.5</v>
@@ -35127,7 +35141,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33">
         <f t="shared" si="2"/>
         <v>12.5</v>
@@ -35162,7 +35176,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34">
         <f t="shared" si="2"/>
         <v>12.5</v>
@@ -35197,7 +35211,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35">
         <f t="shared" si="2"/>
         <v>12.5</v>
@@ -35232,7 +35246,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36">
         <f>A31/2</f>
         <v>12.5</v>
@@ -35267,7 +35281,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37">
         <f t="shared" ref="A37:A46" si="4">A32/2</f>
         <v>6.25</v>
@@ -35302,7 +35316,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38">
         <f t="shared" si="4"/>
         <v>6.25</v>
@@ -35337,7 +35351,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39">
         <f t="shared" si="4"/>
         <v>6.25</v>
@@ -35372,7 +35386,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40">
         <f t="shared" si="4"/>
         <v>6.25</v>
@@ -35407,7 +35421,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41">
         <f t="shared" si="4"/>
         <v>6.25</v>
@@ -35442,7 +35456,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42">
         <f t="shared" si="4"/>
         <v>3.125</v>
@@ -35477,7 +35491,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43">
         <f t="shared" si="4"/>
         <v>3.125</v>
@@ -35512,7 +35526,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44">
         <f t="shared" si="4"/>
         <v>3.125</v>
@@ -35547,7 +35561,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45">
         <f t="shared" si="4"/>
         <v>3.125</v>
@@ -35582,7 +35596,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46">
         <f t="shared" si="4"/>
         <v>3.125</v>
@@ -35617,7 +35631,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>1.33</v>
       </c>
@@ -35651,7 +35665,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>1.33</v>
       </c>
@@ -35685,7 +35699,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>1.33</v>
       </c>
@@ -35719,7 +35733,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>1.33</v>
       </c>
@@ -35753,7 +35767,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>1.33</v>
       </c>
@@ -35787,7 +35801,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>0.26700000000000002</v>
       </c>
@@ -35821,7 +35835,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>0.26700000000000002</v>
       </c>
@@ -35855,7 +35869,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>0.26700000000000002</v>
       </c>
@@ -35889,7 +35903,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>0.26700000000000002</v>
       </c>
@@ -35923,7 +35937,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>0.26700000000000002</v>
       </c>
@@ -35957,7 +35971,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>0</v>
       </c>
@@ -35991,7 +36005,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>0</v>
       </c>
@@ -36025,7 +36039,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>0</v>
       </c>
@@ -36059,7 +36073,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>0</v>
       </c>
@@ -36093,7 +36107,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>0</v>
       </c>
@@ -36136,18 +36150,18 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5DF7757-9133-4402-B2A6-D3896233E79E}">
   <dimension ref="A1:AP73"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7265625" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="14.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.81640625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="12" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5703125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.54296875" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="12" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="14" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>66</v>
       </c>
@@ -36179,7 +36193,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>800</v>
       </c>
@@ -36213,7 +36227,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>800</v>
       </c>
@@ -36239,15 +36253,15 @@
         <v>71</v>
       </c>
       <c r="I3">
-        <f t="shared" ref="I3:I6" si="0">B3*10</f>
+        <f>B3*10</f>
         <v>3184.5878136200699</v>
       </c>
       <c r="J3">
-        <f t="shared" ref="J3:J64" si="1">A3/10</f>
+        <f t="shared" ref="J3:J64" si="0">A3/10</f>
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>800</v>
       </c>
@@ -36273,15 +36287,15 @@
         <v>71</v>
       </c>
       <c r="I4">
+        <f>B4*10</f>
+        <v>3187.5357142857097</v>
+      </c>
+      <c r="J4">
         <f t="shared" si="0"/>
-        <v>3187.5357142857097</v>
-      </c>
-      <c r="J4">
-        <f t="shared" si="1"/>
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>800</v>
       </c>
@@ -36307,15 +36321,15 @@
         <v>71</v>
       </c>
       <c r="I5">
+        <f>B5*10</f>
+        <v>3299.5910780669101</v>
+      </c>
+      <c r="J5">
         <f t="shared" si="0"/>
-        <v>3299.5910780669101</v>
-      </c>
-      <c r="J5">
-        <f t="shared" si="1"/>
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>800</v>
       </c>
@@ -36341,17 +36355,17 @@
         <v>71</v>
       </c>
       <c r="I6">
+        <f>B6*10</f>
+        <v>3189.2831541218602</v>
+      </c>
+      <c r="J6">
         <f t="shared" si="0"/>
-        <v>3189.2831541218602</v>
-      </c>
-      <c r="J6">
-        <f t="shared" si="1"/>
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
-        <f>A2/2</f>
+        <f t="shared" ref="A7:A12" si="1">A2/2</f>
         <v>400</v>
       </c>
       <c r="B7">
@@ -36380,13 +36394,13 @@
         <v>1968.5285714285701</v>
       </c>
       <c r="J7">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A8">
         <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A8">
-        <f>A3/2</f>
         <v>400</v>
       </c>
       <c r="B8">
@@ -36415,13 +36429,13 @@
         <v>1970.7714285714201</v>
       </c>
       <c r="J8">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A9">
         <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A9">
-        <f>A4/2</f>
         <v>400</v>
       </c>
       <c r="B9">
@@ -36450,13 +36464,13 @@
         <v>1973.19285714285</v>
       </c>
       <c r="J9">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A10">
         <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A10">
-        <f>A5/2</f>
         <v>400</v>
       </c>
       <c r="B10">
@@ -36485,13 +36499,13 @@
         <v>1973.2249999999999</v>
       </c>
       <c r="J10">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A11">
         <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A11">
-        <f>A6/2</f>
         <v>400</v>
       </c>
       <c r="B11">
@@ -36520,13 +36534,13 @@
         <v>1973.4035714285701</v>
       </c>
       <c r="J11">
+        <f t="shared" si="0"/>
+        <v>40</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A12">
         <f t="shared" si="1"/>
-        <v>40</v>
-      </c>
-    </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A12">
-        <f t="shared" ref="A12" si="3">A7/2</f>
         <v>200</v>
       </c>
       <c r="B12">
@@ -36555,11 +36569,11 @@
         <v>1036.7071428571401</v>
       </c>
       <c r="J12">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <f>A9/2</f>
         <v>200</v>
@@ -36590,11 +36604,11 @@
         <v>1031.9572953736599</v>
       </c>
       <c r="J13">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <f>A10/2</f>
         <v>200</v>
@@ -36625,11 +36639,11 @@
         <v>1041.3333333333301</v>
       </c>
       <c r="J14">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15">
         <f>A11/2</f>
         <v>200</v>
@@ -36660,11 +36674,11 @@
         <v>984.10714285714198</v>
       </c>
       <c r="J15">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>100</v>
       </c>
@@ -36694,11 +36708,11 @@
         <v>468.12857142857098</v>
       </c>
       <c r="J16">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <f>A13/2</f>
         <v>100</v>
@@ -36729,11 +36743,11 @@
         <v>479.620071684587</v>
       </c>
       <c r="J17">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <f>A14/2</f>
         <v>100</v>
@@ -36764,11 +36778,11 @@
         <v>506.621428571428</v>
       </c>
       <c r="J18">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <f>A15/2</f>
         <v>100</v>
@@ -36799,11 +36813,11 @@
         <v>483.19354838709597</v>
       </c>
       <c r="J19">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>100</v>
       </c>
@@ -36833,11 +36847,11 @@
         <v>485.78494623655899</v>
       </c>
       <c r="J20">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -36867,11 +36881,11 @@
         <v>494.82499999999902</v>
       </c>
       <c r="J21">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>100</v>
       </c>
@@ -36901,11 +36915,11 @@
         <v>493.11827956989202</v>
       </c>
       <c r="J22">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>100</v>
       </c>
@@ -36935,11 +36949,11 @@
         <v>472.69395017793602</v>
       </c>
       <c r="J23">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>100</v>
       </c>
@@ -36969,11 +36983,11 @@
         <v>474.875</v>
       </c>
       <c r="J24">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>10</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>50</v>
       </c>
@@ -36999,15 +37013,15 @@
         <v>72</v>
       </c>
       <c r="I25">
-        <f t="shared" ref="I25:I61" si="4">B25/10</f>
+        <f t="shared" ref="I25:I61" si="3">B25/10</f>
         <v>269.68494623655903</v>
       </c>
       <c r="J25">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <f>A16/2</f>
         <v>50</v>
@@ -37034,15 +37048,15 @@
         <v>72</v>
       </c>
       <c r="I26">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>267.59239130434696</v>
       </c>
       <c r="J26">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <f>A17/2</f>
         <v>50</v>
@@ -37069,15 +37083,15 @@
         <v>72</v>
       </c>
       <c r="I27">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>270.60627306273</v>
       </c>
       <c r="J27">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <f>A18/2</f>
         <v>50</v>
@@ -37104,15 +37118,15 @@
         <v>72</v>
       </c>
       <c r="I28">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>271.18709677419304</v>
       </c>
       <c r="J28">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <f>A19/2</f>
         <v>50</v>
@@ -37139,17 +37153,17 @@
         <v>72</v>
       </c>
       <c r="I29">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>271.17553648068599</v>
       </c>
       <c r="J29">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>5</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
-        <f t="shared" ref="A30:A49" si="5">A25/2</f>
+        <f t="shared" ref="A30:A49" si="4">A25/2</f>
         <v>25</v>
       </c>
       <c r="B30">
@@ -37174,17 +37188,17 @@
         <v>72</v>
       </c>
       <c r="I30">
+        <f t="shared" si="3"/>
+        <v>140.27204301075201</v>
+      </c>
+      <c r="J30">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A31">
         <f t="shared" si="4"/>
-        <v>140.27204301075201</v>
-      </c>
-      <c r="J30">
-        <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A31">
-        <f t="shared" si="5"/>
         <v>25</v>
       </c>
       <c r="B31">
@@ -37209,17 +37223,17 @@
         <v>72</v>
       </c>
       <c r="I31">
+        <f t="shared" si="3"/>
+        <v>140.094244604316</v>
+      </c>
+      <c r="J31">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A32">
         <f t="shared" si="4"/>
-        <v>140.094244604316</v>
-      </c>
-      <c r="J31">
-        <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A32">
-        <f t="shared" si="5"/>
         <v>25</v>
       </c>
       <c r="B32">
@@ -37244,17 +37258,17 @@
         <v>72</v>
       </c>
       <c r="I32">
+        <f t="shared" si="3"/>
+        <v>141.59018181818101</v>
+      </c>
+      <c r="J32">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A33">
         <f t="shared" si="4"/>
-        <v>141.59018181818101</v>
-      </c>
-      <c r="J32">
-        <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A33">
-        <f t="shared" si="5"/>
         <v>25</v>
       </c>
       <c r="B33">
@@ -37279,17 +37293,17 @@
         <v>72</v>
       </c>
       <c r="I33">
+        <f t="shared" si="3"/>
+        <v>135.23273381294899</v>
+      </c>
+      <c r="J33">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A34">
         <f t="shared" si="4"/>
-        <v>135.23273381294899</v>
-      </c>
-      <c r="J33">
-        <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A34">
-        <f t="shared" si="5"/>
         <v>25</v>
       </c>
       <c r="B34">
@@ -37314,17 +37328,17 @@
         <v>72</v>
       </c>
       <c r="I34">
+        <f t="shared" si="3"/>
+        <v>140.043589743589</v>
+      </c>
+      <c r="J34">
+        <f t="shared" si="0"/>
+        <v>2.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A35">
         <f t="shared" si="4"/>
-        <v>140.043589743589</v>
-      </c>
-      <c r="J34">
-        <f t="shared" si="1"/>
-        <v>2.5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A35">
-        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="B35">
@@ -37349,17 +37363,17 @@
         <v>72</v>
       </c>
       <c r="I35">
+        <f t="shared" si="3"/>
+        <v>71.853928571428611</v>
+      </c>
+      <c r="J35">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A36">
         <f t="shared" si="4"/>
-        <v>71.853928571428611</v>
-      </c>
-      <c r="J35">
-        <f t="shared" si="1"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A36">
-        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="B36">
@@ -37384,17 +37398,17 @@
         <v>72</v>
       </c>
       <c r="I36">
+        <f t="shared" si="3"/>
+        <v>63.469999999999899</v>
+      </c>
+      <c r="J36">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A37">
         <f t="shared" si="4"/>
-        <v>63.469999999999899</v>
-      </c>
-      <c r="J36">
-        <f t="shared" si="1"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A37">
-        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="B37">
@@ -37419,17 +37433,17 @@
         <v>72</v>
       </c>
       <c r="I37">
+        <f t="shared" si="3"/>
+        <v>72.856390977443596</v>
+      </c>
+      <c r="J37">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A38">
         <f t="shared" si="4"/>
-        <v>72.856390977443596</v>
-      </c>
-      <c r="J37">
-        <f t="shared" si="1"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A38">
-        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="B38">
@@ -37454,17 +37468,17 @@
         <v>72</v>
       </c>
       <c r="I38">
+        <f t="shared" si="3"/>
+        <v>72.7498207885304</v>
+      </c>
+      <c r="J38">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A39">
         <f t="shared" si="4"/>
-        <v>72.7498207885304</v>
-      </c>
-      <c r="J38">
-        <f t="shared" si="1"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A39">
-        <f t="shared" si="5"/>
         <v>12.5</v>
       </c>
       <c r="B39">
@@ -37489,17 +37503,17 @@
         <v>72</v>
       </c>
       <c r="I39">
+        <f t="shared" si="3"/>
+        <v>73.549795918367295</v>
+      </c>
+      <c r="J39">
+        <f t="shared" si="0"/>
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A40">
         <f t="shared" si="4"/>
-        <v>73.549795918367295</v>
-      </c>
-      <c r="J39">
-        <f t="shared" si="1"/>
-        <v>1.25</v>
-      </c>
-    </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A40">
-        <f t="shared" si="5"/>
         <v>6.25</v>
       </c>
       <c r="B40">
@@ -37524,17 +37538,17 @@
         <v>72</v>
       </c>
       <c r="I40">
+        <f t="shared" si="3"/>
+        <v>40.618699186991805</v>
+      </c>
+      <c r="J40">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A41">
         <f t="shared" si="4"/>
-        <v>40.618699186991805</v>
-      </c>
-      <c r="J40">
-        <f t="shared" si="1"/>
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A41">
-        <f t="shared" si="5"/>
         <v>6.25</v>
       </c>
       <c r="B41">
@@ -37559,17 +37573,17 @@
         <v>72</v>
       </c>
       <c r="I41">
+        <f t="shared" si="3"/>
+        <v>37.939285714285703</v>
+      </c>
+      <c r="J41">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A42">
         <f t="shared" si="4"/>
-        <v>37.939285714285703</v>
-      </c>
-      <c r="J41">
-        <f t="shared" si="1"/>
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A42">
-        <f t="shared" si="5"/>
         <v>6.25</v>
       </c>
       <c r="B42">
@@ -37594,17 +37608,17 @@
         <v>72</v>
       </c>
       <c r="I42">
+        <f t="shared" si="3"/>
+        <v>38.275714285714201</v>
+      </c>
+      <c r="J42">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A43">
         <f t="shared" si="4"/>
-        <v>38.275714285714201</v>
-      </c>
-      <c r="J42">
-        <f t="shared" si="1"/>
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A43">
-        <f t="shared" si="5"/>
         <v>6.25</v>
       </c>
       <c r="B43">
@@ -37629,17 +37643,17 @@
         <v>72</v>
       </c>
       <c r="I43">
+        <f t="shared" si="3"/>
+        <v>38.140377358490504</v>
+      </c>
+      <c r="J43">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A44">
         <f t="shared" si="4"/>
-        <v>38.140377358490504</v>
-      </c>
-      <c r="J43">
-        <f t="shared" si="1"/>
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A44">
-        <f t="shared" si="5"/>
         <v>6.25</v>
       </c>
       <c r="B44">
@@ -37664,17 +37678,17 @@
         <v>72</v>
       </c>
       <c r="I44">
+        <f t="shared" si="3"/>
+        <v>41.509642857142801</v>
+      </c>
+      <c r="J44">
+        <f t="shared" si="0"/>
+        <v>0.625</v>
+      </c>
+    </row>
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A45">
         <f t="shared" si="4"/>
-        <v>41.509642857142801</v>
-      </c>
-      <c r="J44">
-        <f t="shared" si="1"/>
-        <v>0.625</v>
-      </c>
-    </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A45">
-        <f t="shared" si="5"/>
         <v>3.125</v>
       </c>
       <c r="B45">
@@ -37699,17 +37713,17 @@
         <v>72</v>
       </c>
       <c r="I45">
+        <f t="shared" si="3"/>
+        <v>24.399642857142801</v>
+      </c>
+      <c r="J45">
+        <f t="shared" si="0"/>
+        <v>0.3125</v>
+      </c>
+    </row>
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A46">
         <f t="shared" si="4"/>
-        <v>24.399642857142801</v>
-      </c>
-      <c r="J45">
-        <f t="shared" si="1"/>
-        <v>0.3125</v>
-      </c>
-    </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A46">
-        <f t="shared" si="5"/>
         <v>3.125</v>
       </c>
       <c r="B46">
@@ -37734,17 +37748,17 @@
         <v>72</v>
       </c>
       <c r="I46">
+        <f t="shared" si="3"/>
+        <v>21.443629343629301</v>
+      </c>
+      <c r="J46">
+        <f t="shared" si="0"/>
+        <v>0.3125</v>
+      </c>
+    </row>
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A47">
         <f t="shared" si="4"/>
-        <v>21.443629343629301</v>
-      </c>
-      <c r="J46">
-        <f t="shared" si="1"/>
-        <v>0.3125</v>
-      </c>
-    </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A47">
-        <f t="shared" si="5"/>
         <v>3.125</v>
       </c>
       <c r="B47">
@@ -37769,17 +37783,17 @@
         <v>72</v>
       </c>
       <c r="I47">
+        <f t="shared" si="3"/>
+        <v>17.253046594982003</v>
+      </c>
+      <c r="J47">
+        <f t="shared" si="0"/>
+        <v>0.3125</v>
+      </c>
+    </row>
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A48">
         <f t="shared" si="4"/>
-        <v>17.253046594982003</v>
-      </c>
-      <c r="J47">
-        <f t="shared" si="1"/>
-        <v>0.3125</v>
-      </c>
-    </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A48">
-        <f t="shared" si="5"/>
         <v>3.125</v>
       </c>
       <c r="B48">
@@ -37804,17 +37818,17 @@
         <v>72</v>
       </c>
       <c r="I48">
+        <f t="shared" si="3"/>
+        <v>20.827385892116101</v>
+      </c>
+      <c r="J48">
+        <f t="shared" si="0"/>
+        <v>0.3125</v>
+      </c>
+    </row>
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
+      <c r="A49">
         <f t="shared" si="4"/>
-        <v>20.827385892116101</v>
-      </c>
-      <c r="J48">
-        <f t="shared" si="1"/>
-        <v>0.3125</v>
-      </c>
-    </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
-      <c r="A49">
-        <f t="shared" si="5"/>
         <v>3.125</v>
       </c>
       <c r="B49">
@@ -37839,15 +37853,15 @@
         <v>72</v>
       </c>
       <c r="I49">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>23.182499999999997</v>
       </c>
       <c r="J49">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.3125</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>1.33</v>
       </c>
@@ -37873,15 +37887,15 @@
         <v>72</v>
       </c>
       <c r="I50">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>13.7113725490196</v>
       </c>
       <c r="J50">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>1.33</v>
       </c>
@@ -37907,15 +37921,15 @@
         <v>72</v>
       </c>
       <c r="I51">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>14.106761565836299</v>
       </c>
       <c r="J51">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>1.33</v>
       </c>
@@ -37941,15 +37955,15 @@
         <v>72</v>
       </c>
       <c r="I52">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>17.3389285714285</v>
       </c>
       <c r="J52">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>1.33</v>
       </c>
@@ -37975,15 +37989,15 @@
         <v>72</v>
       </c>
       <c r="I53">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>14.152049180327799</v>
       </c>
       <c r="J53">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>1.33</v>
       </c>
@@ -38009,15 +38023,15 @@
         <v>72</v>
       </c>
       <c r="I54">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>14.301433691756198</v>
       </c>
       <c r="J54">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>0.26700000000000002</v>
       </c>
@@ -38043,15 +38057,15 @@
         <v>72</v>
       </c>
       <c r="I55">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>7.8323420074349404</v>
       </c>
       <c r="J55">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>0.26700000000000002</v>
       </c>
@@ -38077,15 +38091,15 @@
         <v>72</v>
       </c>
       <c r="I56">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>7.0706093189964196</v>
       </c>
       <c r="J56">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>0.26700000000000002</v>
       </c>
@@ -38111,15 +38125,15 @@
         <v>72</v>
       </c>
       <c r="I57">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>7.0609442060085801</v>
       </c>
       <c r="J57">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>0.26700000000000002</v>
       </c>
@@ -38145,15 +38159,15 @@
         <v>72</v>
       </c>
       <c r="I58">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>4.6810714285714194</v>
       </c>
       <c r="J58">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>0.26700000000000002</v>
       </c>
@@ -38179,15 +38193,15 @@
         <v>72</v>
       </c>
       <c r="I59">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>5.1722846441947503</v>
       </c>
       <c r="J59">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>0</v>
       </c>
@@ -38213,15 +38227,15 @@
         <v>72</v>
       </c>
       <c r="I60">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>3.6587813620071699</v>
       </c>
       <c r="J60">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>0</v>
       </c>
@@ -38247,15 +38261,15 @@
         <v>72</v>
       </c>
       <c r="I61">
-        <f t="shared" si="4"/>
+        <f t="shared" si="3"/>
         <v>2.4223628691983103</v>
       </c>
       <c r="J61">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="62" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>0</v>
       </c>
@@ -38281,15 +38295,15 @@
         <v>72</v>
       </c>
       <c r="I62">
-        <f t="shared" ref="I62:I64" si="6">B62/10</f>
+        <f>B62/10</f>
         <v>3.1253571428571401</v>
       </c>
       <c r="J62">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="63" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>0</v>
       </c>
@@ -38315,15 +38329,15 @@
         <v>72</v>
       </c>
       <c r="I63">
-        <f t="shared" si="6"/>
+        <f>B63/10</f>
         <v>3.9516363636363598</v>
       </c>
       <c r="J63">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="64" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="64" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>0</v>
       </c>
@@ -38349,15 +38363,15 @@
         <v>72</v>
       </c>
       <c r="I64">
-        <f t="shared" si="6"/>
+        <f>B64/10</f>
         <v>4.4465949820788504</v>
       </c>
       <c r="J64">
-        <f t="shared" si="1"/>
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
     </row>
-    <row r="73" spans="42:42" x14ac:dyDescent="0.25">
+    <row r="73" spans="42:42" x14ac:dyDescent="0.35">
       <c r="AP73" t="s">
         <v>75</v>
       </c>
@@ -38371,13 +38385,13 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{79646366-F568-4C19-B1C0-77B178208506}">
   <dimension ref="A1:AJ69"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="13.7109375" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="21.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="13.7265625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="21.453125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A1" t="s">
         <v>66</v>
       </c>
@@ -38409,7 +38423,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A2">
         <v>800</v>
       </c>
@@ -38443,7 +38457,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>800</v>
       </c>
@@ -38477,7 +38491,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>800</v>
       </c>
@@ -38511,7 +38525,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>800</v>
       </c>
@@ -38545,7 +38559,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>800</v>
       </c>
@@ -38579,9 +38593,9 @@
         <v>80</v>
       </c>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A7">
-        <f>A2/2</f>
+        <f t="shared" ref="A7:A12" si="2">A2/2</f>
         <v>400</v>
       </c>
       <c r="B7">
@@ -38614,9 +38628,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A8">
-        <f>A3/2</f>
+        <f t="shared" si="2"/>
         <v>400</v>
       </c>
       <c r="B8">
@@ -38649,9 +38663,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A9">
-        <f>A4/2</f>
+        <f t="shared" si="2"/>
         <v>400</v>
       </c>
       <c r="B9">
@@ -38684,9 +38698,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A10">
-        <f>A5/2</f>
+        <f t="shared" si="2"/>
         <v>400</v>
       </c>
       <c r="B10">
@@ -38719,9 +38733,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A11">
-        <f>A6/2</f>
+        <f t="shared" si="2"/>
         <v>400</v>
       </c>
       <c r="B11">
@@ -38754,9 +38768,9 @@
         <v>40</v>
       </c>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A12">
-        <f t="shared" ref="A12" si="2">A7/2</f>
+        <f t="shared" si="2"/>
         <v>200</v>
       </c>
       <c r="B12">
@@ -38789,7 +38803,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A13">
         <f>A9/2</f>
         <v>200</v>
@@ -38824,7 +38838,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A14">
         <f>A10/2</f>
         <v>200</v>
@@ -38859,7 +38873,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A15">
         <f>A11/2</f>
         <v>200</v>
@@ -38894,7 +38908,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>200</v>
       </c>
@@ -38928,7 +38942,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>100</v>
       </c>
@@ -38962,7 +38976,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A18">
         <f>A13/2</f>
         <v>100</v>
@@ -38997,7 +39011,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A19">
         <f>A15/2</f>
         <v>100</v>
@@ -39032,7 +39046,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>100</v>
       </c>
@@ -39066,7 +39080,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>100</v>
       </c>
@@ -39100,7 +39114,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>50</v>
       </c>
@@ -39134,7 +39148,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A23">
         <f>A17/2</f>
         <v>50</v>
@@ -39169,7 +39183,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A24">
         <f>A18/2</f>
         <v>50</v>
@@ -39204,7 +39218,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>50</v>
       </c>
@@ -39238,7 +39252,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A26">
         <f>A19/2</f>
         <v>50</v>
@@ -39273,7 +39287,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A27">
         <f t="shared" ref="A27:A36" si="4">A22/2</f>
         <v>25</v>
@@ -39308,7 +39322,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A28">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -39343,7 +39357,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A29">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -39378,7 +39392,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A30">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -39413,7 +39427,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="31" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A31">
         <f t="shared" si="4"/>
         <v>25</v>
@@ -39448,7 +39462,7 @@
         <v>2.5</v>
       </c>
     </row>
-    <row r="32" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A32">
         <f t="shared" si="4"/>
         <v>12.5</v>
@@ -39483,7 +39497,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="33" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A33">
         <f t="shared" si="4"/>
         <v>12.5</v>
@@ -39518,7 +39532,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="34" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A34">
         <f t="shared" si="4"/>
         <v>12.5</v>
@@ -39553,7 +39567,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="35" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A35">
         <f t="shared" si="4"/>
         <v>12.5</v>
@@ -39588,7 +39602,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="36" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="36" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A36">
         <f t="shared" si="4"/>
         <v>12.5</v>
@@ -39623,7 +39637,7 @@
         <v>1.25</v>
       </c>
     </row>
-    <row r="37" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A37">
         <f t="shared" ref="A37:A46" si="5">A32/2</f>
         <v>6.25</v>
@@ -39658,7 +39672,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="38" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="38" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A38">
         <f t="shared" si="5"/>
         <v>6.25</v>
@@ -39693,7 +39707,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="39" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="39" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A39">
         <f t="shared" si="5"/>
         <v>6.25</v>
@@ -39728,7 +39742,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="40" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="40" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A40">
         <f t="shared" si="5"/>
         <v>6.25</v>
@@ -39763,7 +39777,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="41" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A41">
         <f t="shared" si="5"/>
         <v>6.25</v>
@@ -39798,7 +39812,7 @@
         <v>0.625</v>
       </c>
     </row>
-    <row r="42" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A42">
         <f t="shared" si="5"/>
         <v>3.125</v>
@@ -39833,7 +39847,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="43" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A43">
         <f t="shared" si="5"/>
         <v>3.125</v>
@@ -39868,7 +39882,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="44" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A44">
         <f t="shared" si="5"/>
         <v>3.125</v>
@@ -39903,7 +39917,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="45" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="45" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A45">
         <f t="shared" si="5"/>
         <v>3.125</v>
@@ -39938,7 +39952,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="46" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A46">
         <f t="shared" si="5"/>
         <v>3.125</v>
@@ -39973,7 +39987,7 @@
         <v>0.3125</v>
       </c>
     </row>
-    <row r="47" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>1.33</v>
       </c>
@@ -40007,7 +40021,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="48" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>1.33</v>
       </c>
@@ -40041,7 +40055,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="49" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="49" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>1.33</v>
       </c>
@@ -40075,7 +40089,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="50" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="50" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>1.33</v>
       </c>
@@ -40109,7 +40123,7 @@
         <v>0.13300000000000001</v>
       </c>
     </row>
-    <row r="51" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="51" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>0.26700000000000002</v>
       </c>
@@ -40143,7 +40157,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="52" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>0.26700000000000002</v>
       </c>
@@ -40177,7 +40191,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="53" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>0.26700000000000002</v>
       </c>
@@ -40211,7 +40225,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="54" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>0.26700000000000002</v>
       </c>
@@ -40245,7 +40259,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="55" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>0.26700000000000002</v>
       </c>
@@ -40279,7 +40293,7 @@
         <v>2.6700000000000002E-2</v>
       </c>
     </row>
-    <row r="56" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="56" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>0</v>
       </c>
@@ -40313,7 +40327,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="57" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>0</v>
       </c>
@@ -40347,7 +40361,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="58" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>0</v>
       </c>
@@ -40381,7 +40395,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="59" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>0</v>
       </c>
@@ -40415,7 +40429,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="60" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:10" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>0</v>
       </c>
@@ -40449,7 +40463,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="61" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:10" x14ac:dyDescent="0.35">
       <c r="I61">
         <f t="shared" si="3"/>
         <v>0</v>
@@ -40459,7 +40473,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="69" spans="36:36" x14ac:dyDescent="0.25">
+    <row r="69" spans="36:36" x14ac:dyDescent="0.35">
       <c r="AJ69" t="s">
         <v>75</v>
       </c>

</xml_diff>